<commit_message>
deploy: main → 811ad7a3a5c9c6ac1ef5bfb217739b12d4b18483
</commit_message>
<xml_diff>
--- a/CodeSystem-assessmentcategory-cs.xlsx
+++ b/CodeSystem-assessmentcategory-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.3.3</t>
+    <t>0.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-09T07:52:45+00:00</t>
+    <t>2026-10-12T12:51:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → ee4dd0b5f6eb5e7c996226b414bf267e817e428e
</commit_message>
<xml_diff>
--- a/CodeSystem-assessmentcategory-cs.xlsx
+++ b/CodeSystem-assessmentcategory-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.5.0</t>
+    <t>0.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-12T13:38:08+00:00</t>
+    <t>2026-10-15T17:10:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → f9b06e3e936c5f9300cc63ab59951f19cc1ba45e
</commit_message>
<xml_diff>
--- a/CodeSystem-assessmentcategory-cs.xlsx
+++ b/CodeSystem-assessmentcategory-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.7.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T18:03:33+00:00</t>
+    <t>2026-10-26T15:58:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>